<commit_message>
fix: update market sweep Excel files for Brazil, France, Poland, and Spain
</commit_message>
<xml_diff>
--- a/data/market-sweeps/France.xlsx
+++ b/data/market-sweeps/France.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -118,6 +118,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -551,7 +554,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F2" s="7" t="n"/>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>FR0010285965</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -579,7 +586,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F3" s="7" t="n"/>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>FR0013341781</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -607,7 +618,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F4" s="7" t="n"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>FR0010557264</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -635,7 +650,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F5" s="7" t="n"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>FR0004040608</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -663,7 +682,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F6" s="7" t="n"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>FR0013185857</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -691,7 +714,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>FR0012333284</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -719,7 +746,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F8" s="7" t="n"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120404</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -747,7 +778,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F9" s="7" t="n"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>FR0000076655</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -775,7 +810,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F10" s="7" t="n"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>FR0011184241</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -803,7 +842,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F11" s="7" t="n"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>FR0010340141</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -831,7 +874,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F12" s="7" t="n"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>FR0014005AC9</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -859,7 +906,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F13" s="7" t="n"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>FR001400J770</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -887,7 +938,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F14" s="7" t="n"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120073</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -915,7 +970,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F15" s="7" t="n"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>NL0000235190</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -943,7 +1002,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F16" s="7" t="n"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>FR0000053027</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -971,7 +1034,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F17" s="7" t="n"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>FR0010220475</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -999,7 +1066,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F18" s="7" t="n"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>FR0000053837</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1027,7 +1098,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F19" s="7" t="n"/>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>FR0000033219</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1055,7 +1130,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F20" s="7" t="n"/>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>FR0000071946</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1083,7 +1162,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F21" s="7" t="n"/>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>FR0004125920</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1111,7 +1194,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F22" s="7" t="n"/>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>FR0014005AL0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1139,7 +1226,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F23" s="7" t="n"/>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>LU0569974404</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1167,7 +1258,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F24" s="7" t="n"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>FR0014003U94</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1195,7 +1290,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F25" s="7" t="n"/>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>LU1598757687</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1223,7 +1322,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F26" s="7" t="n"/>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>FR0010313833</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1251,7 +1354,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F27" s="7" t="n"/>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>FR001400X2S4</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1279,7 +1386,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F28" s="7" t="n"/>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>FR0000063737</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1307,7 +1418,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F29" s="7" t="n"/>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120628</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1335,7 +1450,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F30" s="7" t="n"/>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>FR0011040500</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1363,7 +1482,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F31" s="7" t="n"/>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>FR0000035164</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1391,7 +1514,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F32" s="7" t="n"/>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120966</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1419,7 +1546,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F33" s="7" t="n"/>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>FR0000074072</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1447,7 +1578,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F34" s="7" t="n"/>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>FR0013280286</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1475,7 +1610,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F35" s="7" t="n"/>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>FR0000131104</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1503,7 +1642,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F36" s="7" t="n"/>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>FR0000061129</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1531,7 +1674,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F37" s="7" t="n"/>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>FR0000039299</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1559,7 +1706,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F38" s="7" t="n"/>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>FR0000063935</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -1587,7 +1738,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F39" s="7" t="n"/>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120503</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1615,7 +1770,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F40" s="7" t="n"/>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>FR0006174348</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1643,7 +1802,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F41" s="7" t="n"/>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>FR0000061137</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1671,7 +1834,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F42" s="7" t="n"/>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>FR0000125338</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1699,7 +1866,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F43" s="7" t="n"/>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>FR0011648716</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1727,7 +1898,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F44" s="7" t="n"/>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>FR0010907956</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -1755,7 +1930,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F45" s="7" t="n"/>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>FR0010828137</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1783,7 +1962,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F46" s="7" t="n"/>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120172</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -1811,7 +1994,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F47" s="7" t="n"/>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>FR001400OKR3</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1839,7 +2026,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F48" s="7" t="n"/>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>FR0010193052</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -1867,7 +2058,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F49" s="7" t="n"/>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>FR0000053506</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1895,7 +2090,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F50" s="7" t="n"/>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>FR0013181864</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -1923,7 +2122,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F51" s="7" t="n"/>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>FR0000130692</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1951,7 +2154,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F52" s="7" t="n"/>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>FR0000130403</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -1979,7 +2186,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F53" s="7" t="n"/>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>FR0013426004</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2007,7 +2218,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F54" s="7" t="n"/>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>FR0010386334</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -2035,7 +2250,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F55" s="7" t="n"/>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>FR0010667147</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2063,7 +2282,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F56" s="7" t="n"/>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>FR0000053324</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -2091,7 +2314,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F57" s="7" t="n"/>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>FR0000062234</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2119,7 +2346,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F58" s="7" t="n"/>
+      <c r="F58" s="8" t="inlineStr">
+        <is>
+          <t>FR0000064578</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2147,7 +2378,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F59" s="7" t="n"/>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>FR0000045072</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2175,7 +2410,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F60" s="7" t="n"/>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120644</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -2203,7 +2442,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F61" s="7" t="n"/>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>FR0014004L86</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2231,7 +2474,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F62" s="7" t="n"/>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>FR0014003TT8</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -2259,7 +2506,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F63" s="7" t="n"/>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>FR0010417345</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2287,7 +2538,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F64" s="7" t="n"/>
+      <c r="F64" s="8" t="inlineStr">
+        <is>
+          <t>FR001400AYG6</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -2315,7 +2570,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F65" s="7" t="n"/>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>FR0000053381</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2343,7 +2602,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F66" s="7" t="n"/>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>FR0010908533</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -2371,7 +2634,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F67" s="7" t="n"/>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>FR0000130452</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2399,7 +2666,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F68" s="7" t="n"/>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>FR0011466069</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -2427,7 +2698,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F69" s="7" t="n"/>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>FR0011950732</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2455,7 +2730,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F70" s="7" t="n"/>
+      <c r="F70" s="8" t="inlineStr">
+        <is>
+          <t>FR0012435121</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -2483,7 +2762,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F71" s="7" t="n"/>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>FR0010208488</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2511,7 +2794,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F72" s="7" t="n"/>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>FR0000131757</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -2567,7 +2854,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F74" s="7" t="n"/>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121667</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -2595,7 +2886,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F75" s="7" t="n"/>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121121</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2623,7 +2918,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F76" s="7" t="n"/>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>FR0014008VX5</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -2651,7 +2950,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F77" s="7" t="n"/>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>FR0014000MR3</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2679,7 +2982,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F78" s="7" t="n"/>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>NL0006294274</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -2707,7 +3014,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F79" s="7" t="n"/>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>FR0010221234</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2735,7 +3046,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F80" s="7" t="n"/>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>FR0000062671</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -2791,7 +3106,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F82" s="7" t="n"/>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>FR0013451333</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -2819,7 +3138,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F83" s="7" t="n"/>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>FR0011665280</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2847,7 +3170,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F84" s="7" t="n"/>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>FR0011476928</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -2875,7 +3202,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F85" s="7" t="n"/>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>FR0014005SB3</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2903,7 +3234,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F86" s="7" t="n"/>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121147</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -2931,7 +3266,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F87" s="7" t="n"/>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>FR0010485268</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2959,7 +3298,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F88" s="7" t="n"/>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>FR0013495298</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -2987,7 +3330,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F89" s="7" t="n"/>
+      <c r="F89" s="8" t="inlineStr">
+        <is>
+          <t>FR0010040865</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3015,7 +3362,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F90" s="7" t="n"/>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t>FR0004163111</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -3043,7 +3394,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F91" s="7" t="n"/>
+      <c r="F91" s="8" t="inlineStr">
+        <is>
+          <t>FR0010533075</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3071,7 +3426,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F92" s="7" t="n"/>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>FR0000066672</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -3099,7 +3458,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F93" s="7" t="n"/>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>FR0011726835</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3127,7 +3490,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F94" s="7" t="n"/>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>FR0000032526</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -3155,7 +3522,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F95" s="7" t="n"/>
+      <c r="F95" s="8" t="inlineStr">
+        <is>
+          <t>FR0000066755</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3183,7 +3554,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F96" s="7" t="n"/>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>FR0000052292</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -3211,7 +3586,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F97" s="7" t="n"/>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>FR0000035081</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3239,7 +3618,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F98" s="7" t="n"/>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>FR0010929125</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -3267,7 +3650,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F99" s="7" t="n"/>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120859</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3295,7 +3682,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F100" s="7" t="n"/>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>FR0010331421</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -3323,7 +3714,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F101" s="7" t="n"/>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>FR0004024222</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -3351,7 +3746,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F102" s="7" t="n"/>
+      <c r="F102" s="8" t="inlineStr">
+        <is>
+          <t>FR0013233012</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -3379,7 +3778,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F103" s="7" t="n"/>
+      <c r="F103" s="8" t="inlineStr">
+        <is>
+          <t>FR0010259150</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3407,7 +3810,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F104" s="7" t="n"/>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>FR0000073298</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -3435,7 +3842,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F105" s="7" t="n"/>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t>FR0000077919</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3463,7 +3874,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F106" s="7" t="n"/>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>FR0004007813</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -3491,7 +3906,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F107" s="7" t="n"/>
+      <c r="F107" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121485</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3519,7 +3938,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F108" s="7" t="n"/>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121964</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -3547,7 +3970,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F109" s="7" t="n"/>
+      <c r="F109" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120321</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3575,7 +4002,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F110" s="7" t="n"/>
+      <c r="F110" s="8" t="inlineStr">
+        <is>
+          <t>FR0000066607</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -3603,7 +4034,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F111" s="7" t="n"/>
+      <c r="F111" s="8" t="inlineStr">
+        <is>
+          <t>FR0000130213</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3631,7 +4066,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F112" s="7" t="n"/>
+      <c r="F112" s="8" t="inlineStr">
+        <is>
+          <t>FR0006864484</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -3659,7 +4098,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F113" s="7" t="n"/>
+      <c r="F113" s="8" t="inlineStr">
+        <is>
+          <t>FR001400SF56</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3687,7 +4130,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F114" s="7" t="n"/>
+      <c r="F114" s="8" t="inlineStr">
+        <is>
+          <t>FR0000065484</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -3715,7 +4162,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F115" s="7" t="n"/>
+      <c r="F115" s="8" t="inlineStr">
+        <is>
+          <t>FR0010307819</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -3743,7 +4194,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F116" s="7" t="n"/>
+      <c r="F116" s="8" t="inlineStr">
+        <is>
+          <t>FR0014009YQ1</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -3771,7 +4226,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F117" s="7" t="n"/>
+      <c r="F117" s="8" t="inlineStr">
+        <is>
+          <t>FR0004156297</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -3799,7 +4258,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F118" s="7" t="n"/>
+      <c r="F118" s="8" t="inlineStr">
+        <is>
+          <t>FR0000050353</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -3827,7 +4290,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F119" s="7" t="n"/>
+      <c r="F119" s="8" t="inlineStr">
+        <is>
+          <t>FR0004170017</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3883,7 +4350,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F121" s="7" t="n"/>
+      <c r="F121" s="8" t="inlineStr">
+        <is>
+          <t>FR0000038242</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3911,7 +4382,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F122" s="7" t="n"/>
+      <c r="F122" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121014</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -3939,7 +4414,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F123" s="7" t="n"/>
+      <c r="F123" s="8" t="inlineStr">
+        <is>
+          <t>FR0013153541</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3967,7 +4446,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F124" s="7" t="n"/>
+      <c r="F124" s="8" t="inlineStr">
+        <is>
+          <t>FR0000038606</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -3995,7 +4478,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F125" s="7" t="n"/>
+      <c r="F125" s="8" t="inlineStr">
+        <is>
+          <t>MA0000011488</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4023,7 +4510,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F126" s="7" t="n"/>
+      <c r="F126" s="8" t="inlineStr">
+        <is>
+          <t>FR0000051070</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -4051,7 +4542,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F127" s="7" t="n"/>
+      <c r="F127" s="8" t="inlineStr">
+        <is>
+          <t>FR0011742329</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -4079,7 +4574,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F128" s="7" t="n"/>
+      <c r="F128" s="8" t="inlineStr">
+        <is>
+          <t>FR0004065605</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -4107,7 +4606,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F129" s="7" t="n"/>
+      <c r="F129" s="8" t="inlineStr">
+        <is>
+          <t>FR0010241638</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -4135,7 +4638,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F130" s="7" t="n"/>
+      <c r="F130" s="8" t="inlineStr">
+        <is>
+          <t>FR0000039620</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -4163,7 +4670,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F131" s="7" t="n"/>
+      <c r="F131" s="8" t="inlineStr">
+        <is>
+          <t>FR0000053225</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -4191,7 +4702,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F132" s="7" t="n"/>
+      <c r="F132" s="8" t="inlineStr">
+        <is>
+          <t>FR001400AJ45</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -4219,7 +4734,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F133" s="7" t="n"/>
+      <c r="F133" s="8" t="inlineStr">
+        <is>
+          <t>FR0013482791</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -4247,7 +4766,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F134" s="7" t="n"/>
+      <c r="F134" s="8" t="inlineStr">
+        <is>
+          <t>FR0011341205</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -4303,7 +4826,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F136" s="7" t="n"/>
+      <c r="F136" s="8" t="inlineStr">
+        <is>
+          <t>FR0004050250</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -4331,7 +4858,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F137" s="7" t="n"/>
+      <c r="F137" s="8" t="inlineStr">
+        <is>
+          <t>FR0000044448</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -4359,7 +4890,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F138" s="7" t="n"/>
+      <c r="F138" s="8" t="inlineStr">
+        <is>
+          <t>FR0010112524</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -4415,7 +4950,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F140" s="7" t="n"/>
+      <c r="F140" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121691</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -4443,7 +4982,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F141" s="7" t="n"/>
+      <c r="F141" s="8" t="inlineStr">
+        <is>
+          <t>FR0000133308</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -4471,7 +5014,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F142" s="7" t="n"/>
+      <c r="F142" s="8" t="inlineStr">
+        <is>
+          <t>FR0014005HJ9</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -4499,7 +5046,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F143" s="7" t="n"/>
+      <c r="F143" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120693</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -4527,7 +5078,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F144" s="7" t="n"/>
+      <c r="F144" s="8" t="inlineStr">
+        <is>
+          <t>FR0000064784</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -4555,7 +5110,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F145" s="7" t="n"/>
+      <c r="F145" s="8" t="inlineStr">
+        <is>
+          <t>FR0000124570</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -4583,7 +5142,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F146" s="7" t="n"/>
+      <c r="F146" s="8" t="inlineStr">
+        <is>
+          <t>FR0000130577</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -4611,7 +5174,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F147" s="7" t="n"/>
+      <c r="F147" s="8" t="inlineStr">
+        <is>
+          <t>FR0004154060</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -4639,7 +5206,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F148" s="7" t="n"/>
+      <c r="F148" s="8" t="inlineStr">
+        <is>
+          <t>FR0000130395</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -4667,7 +5238,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F149" s="7" t="n"/>
+      <c r="F149" s="8" t="inlineStr">
+        <is>
+          <t>FR0000131906</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -4695,7 +5270,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F150" s="7" t="n"/>
+      <c r="F150" s="8" t="inlineStr">
+        <is>
+          <t>FR0010451203</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -4723,7 +5302,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F151" s="7" t="n"/>
+      <c r="F151" s="8" t="inlineStr">
+        <is>
+          <t>FR0000039091</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -4751,7 +5334,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F152" s="7" t="n"/>
+      <c r="F152" s="8" t="inlineStr">
+        <is>
+          <t>FR0013269123</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -4779,7 +5366,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F153" s="7" t="n"/>
+      <c r="F153" s="8" t="inlineStr">
+        <is>
+          <t>FR0000073272</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -4807,7 +5398,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F154" s="7" t="n"/>
+      <c r="F154" s="8" t="inlineStr">
+        <is>
+          <t>FR0000125007</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
@@ -4835,7 +5430,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F155" s="7" t="n"/>
+      <c r="F155" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120578</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -4863,7 +5462,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F156" s="7" t="n"/>
+      <c r="F156" s="8" t="inlineStr">
+        <is>
+          <t>FR0013154002</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -4891,7 +5494,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F157" s="7" t="n"/>
+      <c r="F157" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120107</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -4919,7 +5526,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F158" s="7" t="n"/>
+      <c r="F158" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121972</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -4947,7 +5558,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F159" s="7" t="n"/>
+      <c r="F159" s="8" t="inlineStr">
+        <is>
+          <t>FR0010411983</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -4975,7 +5590,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F160" s="7" t="n"/>
+      <c r="F160" s="8" t="inlineStr">
+        <is>
+          <t>FR0000039139</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -5003,12 +5622,16 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F161" s="7" t="n"/>
+      <c r="F161" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121709</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>SES Imagotag</t>
+          <t>VusionGroup</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -5031,7 +5654,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F162" s="7" t="n"/>
+      <c r="F162" s="8" t="inlineStr">
+        <is>
+          <t>FR0010282822</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -5059,7 +5686,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F163" s="7" t="n"/>
+      <c r="F163" s="8" t="inlineStr">
+        <is>
+          <t>LU0088087324</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -5087,7 +5718,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F164" s="7" t="n"/>
+      <c r="F164" s="8" t="inlineStr">
+        <is>
+          <t>FR0013006558</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -5143,7 +5778,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F166" s="7" t="n"/>
+      <c r="F166" s="8" t="inlineStr">
+        <is>
+          <t>FR0013214145</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -5171,7 +5810,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F167" s="7" t="n"/>
+      <c r="F167" s="8" t="inlineStr">
+        <is>
+          <t>FR0000130809</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -5199,7 +5842,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F168" s="7" t="n"/>
+      <c r="F168" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121220</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -5227,7 +5874,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F169" s="7" t="n"/>
+      <c r="F169" s="8" t="inlineStr">
+        <is>
+          <t>FR0013227113</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -5255,7 +5906,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F170" s="7" t="n"/>
+      <c r="F170" s="8" t="inlineStr">
+        <is>
+          <t>FR0013379484</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -5283,7 +5938,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F171" s="7" t="n"/>
+      <c r="F171" s="8" t="inlineStr">
+        <is>
+          <t>FR0000050809</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -5311,7 +5970,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F172" s="7" t="n"/>
+      <c r="F172" s="8" t="inlineStr">
+        <is>
+          <t>FR0012757854</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -5339,7 +6002,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F173" s="7" t="n"/>
+      <c r="F173" s="8" t="inlineStr">
+        <is>
+          <t>FR0000076028</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -5367,7 +6034,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F174" s="7" t="n"/>
+      <c r="F174" s="8" t="inlineStr">
+        <is>
+          <t>NL0010877643</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -5395,7 +6066,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F175" s="7" t="n"/>
+      <c r="F175" s="8" t="inlineStr">
+        <is>
+          <t>NL0000226223</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -5423,7 +6098,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F176" s="7" t="n"/>
+      <c r="F176" s="8" t="inlineStr">
+        <is>
+          <t>FR0004180578</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -5479,7 +6158,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F178" s="7" t="n"/>
+      <c r="F178" s="8" t="inlineStr">
+        <is>
+          <t>NL0014559478</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -5507,7 +6190,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F179" s="7" t="n"/>
+      <c r="F179" s="8" t="inlineStr">
+        <is>
+          <t>FR0000051807</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -5535,7 +6222,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F180" s="7" t="n"/>
+      <c r="F180" s="8" t="inlineStr">
+        <is>
+          <t>FR0000054900</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -5563,7 +6254,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F181" s="7" t="n"/>
+      <c r="F181" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121329</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -5591,7 +6286,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F182" s="7" t="n"/>
+      <c r="F182" s="8" t="inlineStr">
+        <is>
+          <t>FR0013230612</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -5619,7 +6318,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F183" s="7" t="n"/>
+      <c r="F183" s="8" t="inlineStr">
+        <is>
+          <t>FR0000120271</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -5647,7 +6350,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F184" s="7" t="n"/>
+      <c r="F184" s="8" t="inlineStr">
+        <is>
+          <t>FR0005691656</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -5675,7 +6382,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F185" s="7" t="n"/>
+      <c r="F185" s="8" t="inlineStr">
+        <is>
+          <t>FR0000054470</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -5703,7 +6414,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F186" s="7" t="n"/>
+      <c r="F186" s="8" t="inlineStr">
+        <is>
+          <t>FR0013326246</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -5731,7 +6446,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F187" s="7" t="n"/>
+      <c r="F187" s="8" t="inlineStr">
+        <is>
+          <t>FR0013176526</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -5759,7 +6478,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F188" s="7" t="n"/>
+      <c r="F188" s="8" t="inlineStr">
+        <is>
+          <t>FR0013506730</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
@@ -5787,7 +6510,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F189" s="7" t="n"/>
+      <c r="F189" s="8" t="inlineStr">
+        <is>
+          <t>FR0004056851</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -5815,7 +6542,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F190" s="7" t="n"/>
+      <c r="F190" s="8" t="inlineStr">
+        <is>
+          <t>FR0000124141</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
@@ -5843,7 +6574,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F191" s="7" t="n"/>
+      <c r="F191" s="8" t="inlineStr">
+        <is>
+          <t>FR0013447729</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -5871,7 +6606,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F192" s="7" t="n"/>
+      <c r="F192" s="8" t="inlineStr">
+        <is>
+          <t>FR0010291245</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
@@ -5899,7 +6638,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F193" s="7" t="n"/>
+      <c r="F193" s="8" t="inlineStr">
+        <is>
+          <t>FR0004186856</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -5927,7 +6670,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F194" s="7" t="n"/>
+      <c r="F194" s="8" t="inlineStr">
+        <is>
+          <t>FR0000031775</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -5955,7 +6702,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F195" s="7" t="n"/>
+      <c r="F195" s="8" t="inlineStr">
+        <is>
+          <t>FR0000125486</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -5983,7 +6734,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F196" s="7" t="n"/>
+      <c r="F196" s="8" t="inlineStr">
+        <is>
+          <t>FR0000031577</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
@@ -6011,7 +6766,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F197" s="7" t="n"/>
+      <c r="F197" s="8" t="inlineStr">
+        <is>
+          <t>FR0000127771</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -6039,7 +6798,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F198" s="7" t="n"/>
+      <c r="F198" s="8" t="inlineStr">
+        <is>
+          <t>FR0011995588</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
@@ -6067,7 +6830,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F199" s="7" t="n"/>
+      <c r="F199" s="8" t="inlineStr">
+        <is>
+          <t>FR0004045847</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -6095,7 +6862,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F200" s="7" t="n"/>
+      <c r="F200" s="8" t="inlineStr">
+        <is>
+          <t>FR0012532810</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
@@ -6123,7 +6894,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F201" s="7" t="n"/>
+      <c r="F201" s="8" t="inlineStr">
+        <is>
+          <t>FR0013357621</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -6151,7 +6926,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F202" s="7" t="n"/>
+      <c r="F202" s="8" t="inlineStr">
+        <is>
+          <t>FR0000121204</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -6179,7 +6958,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F203" s="7" t="n"/>
+      <c r="F203" s="8" t="inlineStr">
+        <is>
+          <t>FR0011981968</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -6207,7 +6990,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F204" s="7" t="n"/>
+      <c r="F204" s="8" t="inlineStr">
+        <is>
+          <t>BE0974310428</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
@@ -6235,7 +7022,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F205" s="7" t="n"/>
+      <c r="F205" s="8" t="inlineStr">
+        <is>
+          <t>FR0004034072</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -6263,7 +7054,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F206" s="7" t="n"/>
+      <c r="F206" s="8" t="inlineStr">
+        <is>
+          <t>FR0000074759</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -6291,7 +7086,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F207" s="7" t="n"/>
+      <c r="F207" s="8" t="inlineStr">
+        <is>
+          <t>FR0012819381</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -6319,7 +7118,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F208" s="7" t="n"/>
+      <c r="F208" s="8" t="inlineStr">
+        <is>
+          <t>FR0000075442</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
@@ -6347,7 +7150,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F209" s="7" t="n"/>
+      <c r="F209" s="8" t="inlineStr">
+        <is>
+          <t>FR0004155000</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -6375,7 +7182,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F210" s="7" t="n"/>
+      <c r="F210" s="8" t="inlineStr">
+        <is>
+          <t>FR0000036675</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
@@ -6403,7 +7214,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F211" s="7" t="n"/>
+      <c r="F211" s="8" t="inlineStr">
+        <is>
+          <t>FR0012612646</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -6431,7 +7246,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F212" s="7" t="n"/>
+      <c r="F212" s="8" t="inlineStr">
+        <is>
+          <t>FR0000054231</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
@@ -6459,7 +7278,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F213" s="7" t="n"/>
+      <c r="F213" s="8" t="inlineStr">
+        <is>
+          <t>FR0000071797</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -6487,7 +7310,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F214" s="7" t="n"/>
+      <c r="F214" s="8" t="inlineStr">
+        <is>
+          <t>FR0000044471</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
@@ -6515,7 +7342,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F215" s="7" t="n"/>
+      <c r="F215" s="8" t="inlineStr">
+        <is>
+          <t>FR0000060071</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -6543,7 +7374,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F216" s="7" t="n"/>
+      <c r="F216" s="8" t="inlineStr">
+        <is>
+          <t>FR0000032658</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
@@ -6571,7 +7406,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F217" s="7" t="n"/>
+      <c r="F217" s="8" t="inlineStr">
+        <is>
+          <t>FR0013333432</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -6599,7 +7438,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F218" s="7" t="n"/>
+      <c r="F218" s="8" t="inlineStr">
+        <is>
+          <t>FR0014004EC4</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
@@ -6627,7 +7470,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F219" s="7" t="n"/>
+      <c r="F219" s="8" t="inlineStr">
+        <is>
+          <t>FR0004527638</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -6655,7 +7502,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F220" s="7" t="n"/>
+      <c r="F220" s="8" t="inlineStr">
+        <is>
+          <t>FR0000124414</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
@@ -6683,7 +7534,11 @@
           <t>Euronext Paris</t>
         </is>
       </c>
-      <c r="F221" s="7" t="n"/>
+      <c r="F221" s="8" t="inlineStr">
+        <is>
+          <t>FR0000034894</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">

</xml_diff>